<commit_message>
chore: update vietlott results
</commit_message>
<xml_diff>
--- a/Vietlott_Mega_645_Full_Results.xlsx
+++ b/Vietlott_Mega_645_Full_Results.xlsx
@@ -1315,9 +1315,9 @@
   <mergeCells count="15">
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="E4:F4"/>
+    <mergeCell ref="C14:E14"/>
     <mergeCell ref="C11:E11"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="C14:E14"/>
     <mergeCell ref="C13:E13"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="A5:B5"/>
@@ -65497,34 +65497,34 @@
       </c>
       <c r="B1565" s="8" t="inlineStr">
         <is>
-          <t>15/07/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="C1565" s="8" t="inlineStr">
         <is>
-          <t>Thứ 4</t>
+          <t>Thứ 6</t>
         </is>
       </c>
       <c r="D1565" s="9" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E1565" s="9" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F1565" s="9" t="n">
         <v>26</v>
       </c>
       <c r="G1565" s="9" t="n">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="H1565" s="9" t="n">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="I1565" s="9" t="n">
         <v>43</v>
       </c>
       <c r="J1565" s="10" t="n">
-        <v>101885579123</v>
+        <v>86148921500</v>
       </c>
       <c r="K1565" s="8" t="n">
         <v>0</v>

</xml_diff>